<commit_message>
resource depot UI layout
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excel sheets/LocationData.xlsx
+++ b/Assets/Resources/Excel sheets/LocationData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\artem\Desktop\RMIT\RMIT sem 2 2026\GDS6\VANDERBILT\Assets\Resources\Excel sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Scratch\s3841792\VANDERBILT\Assets\Resources\Excel sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A4CEA58-CF7B-487A-93CC-15C6BCE0F506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8EA92B8-E058-4437-96A0-0FC11622D980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3930" yWindow="2130" windowWidth="30570" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
   <si>
     <t>Name</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Residential</t>
   </si>
   <si>
-    <t>Slum</t>
-  </si>
-  <si>
     <t>Airship Dock</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>Hospital</t>
+  </si>
+  <si>
+    <t>ResourceDepot</t>
   </si>
 </sst>
 </file>
@@ -385,13 +385,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="16.54296875" customWidth="1"/>
+    <col min="3" max="3" width="13.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -402,71 +402,101 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C4" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="C7" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="C8" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="C10" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="17" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>